<commit_message>
conf scheduling: fix changing the configuration tab should not crash the read + fix rewards shouldn't undo penalty orange coloring
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
@@ -20,8 +20,83 @@
 </workbook>
 </file>
 
+<file path=xl/comments10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="C3" authorId="0">
+      <text>
+        <t>S028: Securing scalable Hibernate
+  Chad Poe
+  PINNED BY USER</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="C3" authorId="0">
+      <text>
+        <t>S028: Securing scalable Hibernate
+  Chad Poe
+  PINNED BY USER</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="C45" authorId="0">
+      <text>
+        <t>S028: Securing scalable Hibernate
+  Chad Poe
+  PINNED BY USER</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="C3" authorId="0">
+      <text>
+        <t>S028: Securing scalable Hibernate
+  Chad Poe
+  PINNED BY USER</t>
+      </text>
+    </comment>
+    <comment ref="C4" authorId="0">
+      <text>
+        <t>S028: Securing scalable Hibernate
+  Chad Poe
+  PINNED BY USER</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6300" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6351" uniqueCount="479">
   <si>
     <t>Conference name</t>
   </si>
@@ -1770,6 +1845,9 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FCE94F"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -1916,26 +1994,60 @@
       <c r="A3" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="7" t="s">
+        <v>36</v>
+      </c>
       <c r="C3" s="4" t="s">
         <v>478</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
+      <c r="D3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="P3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="S3" s="7" t="s">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells>
@@ -1945,6 +2057,7 @@
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -16707,6 +16820,9 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FCE94F"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -17466,11 +17582,15 @@
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FCE94F"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -21869,11 +21989,15 @@
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FCE94F"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -22020,51 +22144,119 @@
       <c r="A3" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="7" t="s">
+        <v>36</v>
+      </c>
       <c r="C3" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
+      <c r="D3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="P3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="S3" s="7" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="4" ht="15.0" customHeight="true">
       <c r="A4" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" s="7" t="s">
+        <v>36</v>
+      </c>
       <c r="C4" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
+      <c r="D4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="R4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="S4" s="7" t="s">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells>
@@ -22074,11 +22266,15 @@
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FCE94F"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>

</xml_diff>

<commit_message>
conf scheduling: audienceTypes (plural)
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6640" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6641" uniqueCount="528">
   <si>
     <t>Conference name</t>
   </si>
@@ -681,7 +681,7 @@
     <t>Sector tags</t>
   </si>
   <si>
-    <t>Audience type</t>
+    <t>Audience types</t>
   </si>
   <si>
     <t>Audience level</t>
@@ -1687,6 +1687,9 @@
   </si>
   <si>
     <t>Usable sessions</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
   <si>
     <t>S073: Grok distributed Tensorflow
@@ -1703,6 +1706,9 @@
   </si>
   <si>
     <t>Sector tag</t>
+  </si>
+  <si>
+    <t>Audience type</t>
   </si>
   <si>
     <t>1</t>
@@ -2301,7 +2307,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>78</v>
@@ -2459,7 +2465,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>182</v>
+        <v>524</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>78</v>
@@ -2524,7 +2530,7 @@
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -2736,13 +2742,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -2895,7 +2901,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>78</v>
@@ -2960,7 +2966,7 @@
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -18218,6 +18224,24 @@
       </c>
       <c r="E5" s="2" t="n">
         <v>96.0</v>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>108.0</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>18.0</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>180.0</v>
       </c>
     </row>
   </sheetData>
@@ -18400,7 +18424,7 @@
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -19084,7 +19108,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>78</v>
@@ -20978,7 +21002,7 @@
         <v>65</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>65</v>
@@ -23491,7 +23515,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>78</v>
@@ -23556,7 +23580,7 @@
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -23615,7 +23639,7 @@
         <v>65</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>65</v>

</xml_diff>

<commit_message>
conf scheduling: TalkType concept + value range from entity to improve speed
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
@@ -3538,7 +3538,7 @@
       <c r="C3" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -3547,7 +3547,7 @@
       <c r="F3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -3556,7 +3556,7 @@
       <c r="I3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="2" t="s">
         <v>65</v>
       </c>
       <c r="K3" s="2" t="s">
@@ -3565,7 +3565,7 @@
       <c r="L3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="2" t="s">
         <v>65</v>
       </c>
       <c r="N3" s="2" t="s">
@@ -3574,7 +3574,7 @@
       <c r="O3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="P3" s="3" t="s">
+      <c r="P3" s="2" t="s">
         <v>65</v>
       </c>
       <c r="Q3" s="2" t="s">
@@ -3583,7 +3583,7 @@
       <c r="R3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="S3" s="2" t="s">
         <v>65</v>
       </c>
       <c r="T3" s="2" t="s">
@@ -3603,7 +3603,7 @@
       <c r="C4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -3612,7 +3612,7 @@
       <c r="F4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -3621,7 +3621,7 @@
       <c r="I4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="2" t="s">
         <v>65</v>
       </c>
       <c r="K4" s="2" t="s">
@@ -3630,7 +3630,7 @@
       <c r="L4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="2" t="s">
         <v>65</v>
       </c>
       <c r="N4" s="2" t="s">
@@ -3639,7 +3639,7 @@
       <c r="O4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="P4" s="3" t="s">
+      <c r="P4" s="2" t="s">
         <v>65</v>
       </c>
       <c r="Q4" s="2" t="s">
@@ -3648,7 +3648,7 @@
       <c r="R4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="S4" s="3" t="s">
+      <c r="S4" s="2" t="s">
         <v>65</v>
       </c>
       <c r="T4" s="2" t="s">
@@ -3668,7 +3668,7 @@
       <c r="C5" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -3677,7 +3677,7 @@
       <c r="F5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -3686,7 +3686,7 @@
       <c r="I5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -3695,7 +3695,7 @@
       <c r="L5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="N5" s="2" t="s">
@@ -3704,7 +3704,7 @@
       <c r="O5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="P5" s="3" t="s">
+      <c r="P5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="Q5" s="2" t="s">
@@ -3713,7 +3713,7 @@
       <c r="R5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="S5" s="3" t="s">
+      <c r="S5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="T5" s="2" t="s">
@@ -3733,7 +3733,7 @@
       <c r="C6" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E6" s="2" t="s">
@@ -3742,7 +3742,7 @@
       <c r="F6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H6" s="2" t="s">
@@ -3751,7 +3751,7 @@
       <c r="I6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="2" t="s">
         <v>65</v>
       </c>
       <c r="K6" s="2" t="s">
@@ -3760,7 +3760,7 @@
       <c r="L6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M6" s="3" t="s">
+      <c r="M6" s="2" t="s">
         <v>65</v>
       </c>
       <c r="N6" s="2" t="s">
@@ -3769,7 +3769,7 @@
       <c r="O6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="P6" s="3" t="s">
+      <c r="P6" s="2" t="s">
         <v>65</v>
       </c>
       <c r="Q6" s="2" t="s">
@@ -3778,7 +3778,7 @@
       <c r="R6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="S6" s="3" t="s">
+      <c r="S6" s="2" t="s">
         <v>65</v>
       </c>
       <c r="T6" s="2" t="s">
@@ -3801,55 +3801,55 @@
       <c r="D7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F7" s="3" t="s">
+      <c r="E7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="H7" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="I7" s="3" t="s">
+      <c r="H7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>65</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="K7" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="L7" s="3" t="s">
+      <c r="K7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>65</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="N7" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="O7" s="3" t="s">
+      <c r="N7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="O7" s="2" t="s">
         <v>65</v>
       </c>
       <c r="P7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="Q7" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="R7" s="3" t="s">
+      <c r="Q7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="R7" s="2" t="s">
         <v>65</v>
       </c>
       <c r="S7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="T7" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="U7" s="3" t="s">
+      <c r="T7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="U7" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
       <c r="C8" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -3872,7 +3872,7 @@
       <c r="F8" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H8" s="2" t="s">
@@ -3881,7 +3881,7 @@
       <c r="I8" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="2" t="s">
         <v>65</v>
       </c>
       <c r="K8" s="2" t="s">
@@ -3890,7 +3890,7 @@
       <c r="L8" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M8" s="3" t="s">
+      <c r="M8" s="2" t="s">
         <v>65</v>
       </c>
       <c r="N8" s="2" t="s">
@@ -3899,7 +3899,7 @@
       <c r="O8" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="P8" s="3" t="s">
+      <c r="P8" s="2" t="s">
         <v>65</v>
       </c>
       <c r="Q8" s="2" t="s">
@@ -3908,7 +3908,7 @@
       <c r="R8" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="S8" s="3" t="s">
+      <c r="S8" s="2" t="s">
         <v>65</v>
       </c>
       <c r="T8" s="2" t="s">
@@ -3928,7 +3928,7 @@
       <c r="C9" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -3937,7 +3937,7 @@
       <c r="F9" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H9" s="2" t="s">
@@ -3946,7 +3946,7 @@
       <c r="I9" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="J9" s="2" t="s">
         <v>65</v>
       </c>
       <c r="K9" s="2" t="s">
@@ -3955,7 +3955,7 @@
       <c r="L9" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="M9" s="2" t="s">
         <v>65</v>
       </c>
       <c r="N9" s="2" t="s">
@@ -3964,7 +3964,7 @@
       <c r="O9" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="P9" s="3" t="s">
+      <c r="P9" s="2" t="s">
         <v>65</v>
       </c>
       <c r="Q9" s="2" t="s">
@@ -3973,7 +3973,7 @@
       <c r="R9" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="S9" s="3" t="s">
+      <c r="S9" s="2" t="s">
         <v>65</v>
       </c>
       <c r="T9" s="2" t="s">
@@ -3993,7 +3993,7 @@
       <c r="C10" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E10" s="2" t="s">
@@ -4002,7 +4002,7 @@
       <c r="F10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H10" s="2" t="s">
@@ -4011,7 +4011,7 @@
       <c r="I10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="J10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="K10" s="2" t="s">
@@ -4020,7 +4020,7 @@
       <c r="L10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="M10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="N10" s="2" t="s">
@@ -4029,7 +4029,7 @@
       <c r="O10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="P10" s="3" t="s">
+      <c r="P10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="Q10" s="2" t="s">
@@ -4038,7 +4038,7 @@
       <c r="R10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="S10" s="3" t="s">
+      <c r="S10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="T10" s="2" t="s">
@@ -4058,7 +4058,7 @@
       <c r="C11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E11" s="2" t="s">
@@ -4067,7 +4067,7 @@
       <c r="F11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H11" s="2" t="s">
@@ -4076,7 +4076,7 @@
       <c r="I11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="J11" s="2" t="s">
         <v>65</v>
       </c>
       <c r="K11" s="2" t="s">
@@ -4085,7 +4085,7 @@
       <c r="L11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M11" s="3" t="s">
+      <c r="M11" s="2" t="s">
         <v>65</v>
       </c>
       <c r="N11" s="2" t="s">
@@ -4094,7 +4094,7 @@
       <c r="O11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="P11" s="3" t="s">
+      <c r="P11" s="2" t="s">
         <v>65</v>
       </c>
       <c r="Q11" s="2" t="s">
@@ -4103,7 +4103,7 @@
       <c r="R11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="S11" s="3" t="s">
+      <c r="S11" s="2" t="s">
         <v>65</v>
       </c>
       <c r="T11" s="2" t="s">
@@ -4126,55 +4126,55 @@
       <c r="D12" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F12" s="3" t="s">
+      <c r="E12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="H12" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="I12" s="3" t="s">
+      <c r="H12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I12" s="2" t="s">
         <v>65</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="K12" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="L12" s="3" t="s">
+      <c r="K12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L12" s="2" t="s">
         <v>65</v>
       </c>
       <c r="M12" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="N12" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="O12" s="3" t="s">
+      <c r="N12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="O12" s="2" t="s">
         <v>65</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="Q12" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="R12" s="3" t="s">
+      <c r="Q12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="R12" s="2" t="s">
         <v>65</v>
       </c>
       <c r="S12" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="T12" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="U12" s="3" t="s">
+      <c r="T12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="U12" s="2" t="s">
         <v>65</v>
       </c>
     </row>

</xml_diff>

<commit_message>
conf scheduling: increase weight on content conflict and enable some other score rules
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
@@ -1918,7 +1918,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>10</v>
@@ -1940,7 +1940,7 @@
         <v>13</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>14</v>
@@ -1962,7 +1962,7 @@
         <v>17</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>10.0</v>
+        <v>100.0</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>18</v>
@@ -1984,7 +1984,7 @@
         <v>21</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>10.0</v>
+        <v>20.0</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>22</v>
@@ -1995,7 +1995,7 @@
         <v>23</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>10.0</v>
+        <v>20.0</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>24</v>
@@ -2006,7 +2006,7 @@
         <v>25</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>10.0</v>
+        <v>20.0</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>22</v>
@@ -2017,7 +2017,7 @@
         <v>26</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>10.0</v>
+        <v>20.0</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>24</v>
@@ -2028,7 +2028,7 @@
         <v>27</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>10.0</v>
+        <v>20.0</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>28</v>
@@ -2039,7 +2039,7 @@
         <v>29</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>10.0</v>
+        <v>20.0</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>30</v>
@@ -2050,7 +2050,7 @@
         <v>31</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>10.0</v>
+        <v>20.0</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>28</v>
@@ -2061,7 +2061,7 @@
         <v>32</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>10.0</v>
+        <v>20.0</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Extract XLSX common code from conference scheduling example
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
@@ -11,14 +11,16 @@
     <sheet name="Rooms" r:id="rId5" sheetId="3"/>
     <sheet name="Speakers" r:id="rId6" sheetId="4"/>
     <sheet name="Talks" r:id="rId7" sheetId="5"/>
-    <sheet name="Score view" r:id="rId8" sheetId="6"/>
+    <sheet name="Infeasible view" r:id="rId8" sheetId="6"/>
     <sheet name="Rooms view" r:id="rId9" sheetId="7"/>
     <sheet name="Speakers view" r:id="rId10" sheetId="8"/>
     <sheet name="Theme tracks view" r:id="rId11" sheetId="9"/>
     <sheet name="Sectors view" r:id="rId12" sheetId="10"/>
-    <sheet name="Audience type view" r:id="rId13" sheetId="11"/>
-    <sheet name="Audience level view" r:id="rId14" sheetId="12"/>
+    <sheet name="Audience types view" r:id="rId13" sheetId="11"/>
+    <sheet name="Audience levels view" r:id="rId14" sheetId="12"/>
     <sheet name="Contents view" r:id="rId15" sheetId="13"/>
+    <sheet name="Languages view" r:id="rId16" sheetId="14"/>
+    <sheet name="Score view" r:id="rId17" sheetId="15"/>
   </sheets>
 </workbook>
 </file>
@@ -31,9 +33,10 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t>S073: Grok distributed Tensorflow
-  Beth King
-  PINNED BY USER</t>
+        <t xml:space="preserve">S073: Grok distributed Tensorflow
+    Beth King
+PINNED BY USER
+</t>
       </text>
     </comment>
   </commentList>
@@ -48,9 +51,10 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t>S073: Grok distributed Tensorflow
-  Beth King
-  PINNED BY USER</t>
+        <t xml:space="preserve">S073: Grok distributed Tensorflow
+    Beth King
+PINNED BY USER
+</t>
       </text>
     </comment>
   </commentList>
@@ -65,9 +69,28 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t>S073: Grok distributed Tensorflow
-  Beth King
-  PINNED BY USER</t>
+        <t xml:space="preserve">S073: Grok distributed Tensorflow
+    Beth King
+PINNED BY USER
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments14.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="C3" authorId="0">
+      <text>
+        <t xml:space="preserve">S073: Grok distributed Tensorflow
+    Beth King
+PINNED BY USER
+</t>
       </text>
     </comment>
   </commentList>
@@ -82,9 +105,10 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t>S073: Grok distributed Tensorflow
-  Beth King
-  PINNED BY USER</t>
+        <t xml:space="preserve">S073: Grok distributed Tensorflow
+    Beth King
+PINNED BY USER
+</t>
       </text>
     </comment>
   </commentList>
@@ -99,9 +123,10 @@
   <commentList>
     <comment ref="C34" authorId="0">
       <text>
-        <t>S073: Grok distributed Tensorflow
-  Beth King
-  PINNED BY USER</t>
+        <t xml:space="preserve">S073: Grok distributed Tensorflow
+    Beth King
+PINNED BY USER
+</t>
       </text>
     </comment>
   </commentList>
@@ -116,16 +141,18 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t>S073: Grok distributed Tensorflow
-  Beth King
-  PINNED BY USER</t>
+        <t xml:space="preserve">S073: Grok distributed Tensorflow
+    Beth King
+PINNED BY USER
+</t>
       </text>
     </comment>
     <comment ref="C4" authorId="0">
       <text>
-        <t>S073: Grok distributed Tensorflow
-  Beth King
-  PINNED BY USER</t>
+        <t xml:space="preserve">S073: Grok distributed Tensorflow
+    Beth King
+PINNED BY USER
+</t>
       </text>
     </comment>
   </commentList>
@@ -133,7 +160,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6641" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6703" uniqueCount="531">
   <si>
     <t>Conference name</t>
   </si>
@@ -1718,6 +1745,15 @@
   </si>
   <si>
     <t>S073 (level 1)</t>
+  </si>
+  <si>
+    <t>Constraint match</t>
+  </si>
+  <si>
+    <t>Match score</t>
+  </si>
+  <si>
+    <t>Total score</t>
   </si>
 </sst>
 </file>
@@ -1829,6 +1865,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
 </file>
 
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
+<file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
 </file>
@@ -3026,6 +3070,261 @@
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FCE94F"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="9.7109375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="14" max="14" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="16" max="16" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="17" max="17" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="18" max="18" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="19" max="19" width="11.86328125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" ht="15.0" customHeight="true">
+      <c r="A3" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="P3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="S3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>513</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="H1:M1"/>
+    <mergeCell ref="N1:S1"/>
+  </mergeCells>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FCE94F"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="16.8125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="12.296875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.08203125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>530</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -18241,7 +18540,7 @@
         <v>10.0</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>180.0</v>
+        <v>108.0</v>
       </c>
     </row>
   </sheetData>
@@ -18416,7 +18715,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" ht="60.0" customHeight="true">
+    <row r="3" ht="45.0" customHeight="true">
       <c r="A3" s="2" t="s">
         <v>84</v>
       </c>
@@ -18475,7 +18774,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" ht="60.0" customHeight="true">
+    <row r="4" ht="45.0" customHeight="true">
       <c r="A4" s="2" t="s">
         <v>86</v>
       </c>
@@ -18534,7 +18833,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" ht="60.0" customHeight="true">
+    <row r="5" ht="45.0" customHeight="true">
       <c r="A5" s="2" t="s">
         <v>87</v>
       </c>
@@ -18593,7 +18892,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" ht="60.0" customHeight="true">
+    <row r="6" ht="45.0" customHeight="true">
       <c r="A6" s="2" t="s">
         <v>89</v>
       </c>
@@ -18652,7 +18951,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" ht="60.0" customHeight="true">
+    <row r="7" ht="45.0" customHeight="true">
       <c r="A7" s="2" t="s">
         <v>90</v>
       </c>
@@ -18711,7 +19010,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" ht="60.0" customHeight="true">
+    <row r="8" ht="45.0" customHeight="true">
       <c r="A8" s="2" t="s">
         <v>91</v>
       </c>
@@ -18770,7 +19069,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" ht="60.0" customHeight="true">
+    <row r="9" ht="45.0" customHeight="true">
       <c r="A9" s="2" t="s">
         <v>92</v>
       </c>
@@ -18829,7 +19128,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" ht="60.0" customHeight="true">
+    <row r="10" ht="45.0" customHeight="true">
       <c r="A10" s="2" t="s">
         <v>93</v>
       </c>
@@ -18888,7 +19187,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" ht="60.0" customHeight="true">
+    <row r="11" ht="45.0" customHeight="true">
       <c r="A11" s="2" t="s">
         <v>94</v>
       </c>
@@ -18947,7 +19246,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" ht="60.0" customHeight="true">
+    <row r="12" ht="45.0" customHeight="true">
       <c r="A12" s="2" t="s">
         <v>95</v>
       </c>
@@ -19027,24 +19326,43 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.75390625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="10" max="10" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="12" max="12" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="13" max="13" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="14" max="14" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="16" max="16" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="17" max="17" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="18" max="18" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="19" max="19" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="20.0" customWidth="true"/>
+    <col min="3" max="3" width="20.0" customWidth="true"/>
+    <col min="4" max="4" width="20.0" customWidth="true"/>
+    <col min="5" max="5" width="20.0" customWidth="true"/>
+    <col min="6" max="6" width="20.0" customWidth="true"/>
+    <col min="7" max="7" width="20.0" customWidth="true"/>
+    <col min="8" max="8" width="20.0" customWidth="true"/>
+    <col min="9" max="9" width="20.0" customWidth="true"/>
+    <col min="10" max="10" width="20.0" customWidth="true"/>
+    <col min="11" max="11" width="20.0" customWidth="true"/>
+    <col min="12" max="12" width="20.0" customWidth="true"/>
+    <col min="13" max="13" width="20.0" customWidth="true"/>
+    <col min="14" max="14" width="20.0" customWidth="true"/>
+    <col min="15" max="15" width="20.0" customWidth="true"/>
+    <col min="16" max="16" width="20.0" customWidth="true"/>
+    <col min="17" max="17" width="20.0" customWidth="true"/>
+    <col min="18" max="18" width="20.0" customWidth="true"/>
+    <col min="19" max="19" width="20.0" customWidth="true"/>
+    <col min="20" max="20" width="20.0" customWidth="true"/>
+    <col min="21" max="21" width="20.0" customWidth="true"/>
+    <col min="22" max="22" width="20.0" customWidth="true"/>
+    <col min="23" max="23" width="20.0" customWidth="true"/>
+    <col min="24" max="24" width="20.0" customWidth="true"/>
+    <col min="25" max="25" width="20.0" customWidth="true"/>
+    <col min="26" max="26" width="20.0" customWidth="true"/>
+    <col min="27" max="27" width="20.0" customWidth="true"/>
+    <col min="28" max="28" width="20.0" customWidth="true"/>
+    <col min="29" max="29" width="20.0" customWidth="true"/>
+    <col min="30" max="30" width="20.0" customWidth="true"/>
+    <col min="31" max="31" width="20.0" customWidth="true"/>
+    <col min="32" max="32" width="20.0" customWidth="true"/>
+    <col min="33" max="33" width="20.0" customWidth="true"/>
+    <col min="34" max="34" width="20.0" customWidth="true"/>
+    <col min="35" max="35" width="20.0" customWidth="true"/>
+    <col min="36" max="36" width="20.0" customWidth="true"/>
+    <col min="37" max="37" width="20.0" customWidth="true"/>
+    <col min="38" max="38" width="20.0" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Fix typos and drools warning
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
@@ -225,40 +225,40 @@
     <t>Soft reward per 2 talks that have the same timeslot and a different language</t>
   </si>
   <si>
-    <t>Speaker preferred timeslot tag</t>
+    <t>Speaker preferred timeslot tags</t>
   </si>
   <si>
     <t>Soft penalty per missing preferred tag in a talk's timeslot</t>
   </si>
   <si>
-    <t>Speaker undesired timeslot tag</t>
+    <t>Speaker undesired timeslot tags</t>
   </si>
   <si>
     <t>Soft penalty per undesired tag in a talk's timeslot</t>
   </si>
   <si>
-    <t>Talk preferred timeslot tag</t>
-  </si>
-  <si>
-    <t>Talk undesired timeslot tag</t>
-  </si>
-  <si>
-    <t>Speaker preferred room tag</t>
+    <t>Talk preferred timeslot tags</t>
+  </si>
+  <si>
+    <t>Talk undesired timeslot tags</t>
+  </si>
+  <si>
+    <t>Speaker preferred room tags</t>
   </si>
   <si>
     <t>Soft penalty per missing preferred tag in a talk's room</t>
   </si>
   <si>
-    <t>Speaker undesired room tag</t>
+    <t>Speaker undesired room tags</t>
   </si>
   <si>
     <t>Soft penalty per undesired tag in a talk's room</t>
   </si>
   <si>
-    <t>Talk preferred room tag</t>
-  </si>
-  <si>
-    <t>Talk undesired room tag</t>
+    <t>Talk preferred room tags</t>
+  </si>
+  <si>
+    <t>Talk undesired room tags</t>
   </si>
   <si>
     <t>Same day talks</t>
@@ -309,43 +309,43 @@
     <t>Hard penalty per pair of talks with the same speaker in overlapping timeslots</t>
   </si>
   <si>
-    <t>Speaker required timeslot tag</t>
+    <t>Speaker required timeslot tags</t>
   </si>
   <si>
     <t>Hard penalty per missing required tag in a talk's timeslot</t>
   </si>
   <si>
-    <t>Speaker prohibited timeslot tag</t>
+    <t>Speaker prohibited timeslot tags</t>
   </si>
   <si>
     <t>Hard penalty per prohibited tag in a talk's timeslot</t>
   </si>
   <si>
-    <t>Talk required timeslot tag</t>
-  </si>
-  <si>
-    <t>Talk prohibited timeslot tag</t>
-  </si>
-  <si>
-    <t>Speaker required room tag</t>
+    <t>Talk required timeslot tags</t>
+  </si>
+  <si>
+    <t>Talk prohibited timeslot tags</t>
+  </si>
+  <si>
+    <t>Speaker required room tags</t>
   </si>
   <si>
     <t>Hard penalty per missing required tag in a talk's room</t>
   </si>
   <si>
-    <t>Speaker prohibited room tag</t>
+    <t>Speaker prohibited room tags</t>
   </si>
   <si>
     <t>Hard penalty per prohibited tag in a talk's room</t>
   </si>
   <si>
-    <t>Talk required room tag</t>
-  </si>
-  <si>
-    <t>Talk prohibited room tag</t>
-  </si>
-  <si>
-    <t>Talk mutually-exclusive-talks tag</t>
+    <t>Talk required room tags</t>
+  </si>
+  <si>
+    <t>Talk prohibited room tags</t>
+  </si>
+  <si>
+    <t>Talk mutually-exclusive-talks tags</t>
   </si>
   <si>
     <t>Hard penalty per two talks that share the same Mutually exclusive talks tag that are scheduled in overlapping timeslots</t>

</xml_diff>

<commit_message>
Rename numberOfLikes to favoriteCount
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/108talks-18timeslots-10rooms.xlsx
@@ -286,7 +286,7 @@
     <t>Popular talks</t>
   </si>
   <si>
-    <t>Soft penalty per 2 talks where the less popular one (has lower number of likes) is assigned a larger room than the more popular talk</t>
+    <t>Soft penalty per 2 talks where the less popular one (has lower favorite count) is assigned a larger room than the more popular talk</t>
   </si>
   <si>
     <t>Crowd control</t>
@@ -778,7 +778,7 @@
     <t>Prerequisite talks codes</t>
   </si>
   <si>
-    <t>Number of likes</t>
+    <t>Favorite count</t>
   </si>
   <si>
     <t>Crowd control risk</t>
@@ -10867,7 +10867,7 @@
     <col min="18" max="18" width="22.84375" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="31.2734375" customWidth="true" bestFit="true"/>
     <col min="20" max="20" width="26.23046875" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="17.5390625" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="16.25390625" customWidth="true" bestFit="true"/>
     <col min="22" max="22" width="20.140625" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="16.65234375" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.14453125" customWidth="true" bestFit="true"/>

</xml_diff>